<commit_message>
salvataggio dello stato del lavoro al 7 luglio
</commit_message>
<xml_diff>
--- a/ADZ_filtered.xlsx
+++ b/ADZ_filtered.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Domanda1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Domanda 2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Domanda 3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domanda1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domanda 2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domanda 3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -638,202 +638,202 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
+          <t>attività uso della tecnologia</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>scienza</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>misure</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>storytelling</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>geografia</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>coding unplugged</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>attività unplugged</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>decomposizione</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>geometria</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>sviluppo iterativo</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>verifica e correzione</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>ricerca di informazioni</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>pixel art</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>sequenza</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>programmazione</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>coding</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>altre attività</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>aritmetica</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>attività sviluppo contenuti</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>attività ludico-motoria</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>techno-CLIL</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>istruzioni di base</t>
+        </is>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>esecuzione di istruzioni</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>labirinto</t>
+        </is>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>strutture dati</t>
+        </is>
+      </c>
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>lettura codice</t>
+        </is>
+      </c>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>riferimenti topologici</t>
+        </is>
+      </c>
+      <c r="BL2" t="inlineStr">
+        <is>
+          <t>pseudo-linguaggio</t>
+        </is>
+      </c>
+      <c r="BM2" t="inlineStr">
+        <is>
+          <t>intelligenza artificiale</t>
+        </is>
+      </c>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>coding analogico</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr">
+        <is>
+          <t>attività costruzione di mappe</t>
+        </is>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>conversazione collaborativa / collaborazione</t>
+        </is>
+      </c>
+      <c r="BQ2" t="inlineStr">
+        <is>
+          <t>pensiero critico</t>
+        </is>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>pensiero creativo</t>
+        </is>
+      </c>
+      <c r="BS2" t="inlineStr">
+        <is>
+          <t>rianalizzare</t>
+        </is>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>pensiero computazionale</t>
+        </is>
+      </c>
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>risoluzione di problemi</t>
+        </is>
+      </c>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>videotutorial</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>pianificazione</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr">
+        <is>
           <t>uso della tecnologia</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>scienza</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>misure</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>storytelling</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>geografia</t>
-        </is>
-      </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>coding unplugged</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>attività unplugged</t>
-        </is>
-      </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>decomposizione</t>
-        </is>
-      </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>geometria</t>
-        </is>
-      </c>
-      <c r="AT2" t="inlineStr">
-        <is>
-          <t>sviluppo iterativo</t>
-        </is>
-      </c>
-      <c r="AU2" t="inlineStr">
-        <is>
-          <t>verifica e correzione</t>
-        </is>
-      </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>ricerca di informazioni</t>
-        </is>
-      </c>
-      <c r="AW2" t="inlineStr">
-        <is>
-          <t>pixel art</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr">
-        <is>
-          <t>sequenza</t>
-        </is>
-      </c>
-      <c r="AY2" t="inlineStr">
-        <is>
-          <t>programmazione</t>
-        </is>
-      </c>
-      <c r="AZ2" t="inlineStr">
-        <is>
-          <t>coding</t>
-        </is>
-      </c>
-      <c r="BA2" t="inlineStr">
-        <is>
-          <t>altre attività</t>
-        </is>
-      </c>
-      <c r="BB2" t="inlineStr">
-        <is>
-          <t>aritmetica</t>
-        </is>
-      </c>
-      <c r="BC2" t="inlineStr">
-        <is>
-          <t>sviluppo contenuti2</t>
-        </is>
-      </c>
-      <c r="BD2" t="inlineStr">
-        <is>
-          <t>ludico-motoria2</t>
-        </is>
-      </c>
-      <c r="BE2" t="inlineStr">
-        <is>
-          <t>techno-CLIL</t>
-        </is>
-      </c>
-      <c r="BF2" t="inlineStr">
-        <is>
-          <t>istruzioni di base</t>
-        </is>
-      </c>
-      <c r="BG2" t="inlineStr">
-        <is>
-          <t>esecuzione di istruzioni</t>
-        </is>
-      </c>
-      <c r="BH2" t="inlineStr">
-        <is>
-          <t>labirinto</t>
-        </is>
-      </c>
-      <c r="BI2" t="inlineStr">
-        <is>
-          <t>strutture dati</t>
-        </is>
-      </c>
-      <c r="BJ2" t="inlineStr">
-        <is>
-          <t>lettura codice</t>
-        </is>
-      </c>
-      <c r="BK2" t="inlineStr">
-        <is>
-          <t>riferimenti topologici</t>
-        </is>
-      </c>
-      <c r="BL2" t="inlineStr">
-        <is>
-          <t>pseudo-linguaggio</t>
-        </is>
-      </c>
-      <c r="BM2" t="inlineStr">
-        <is>
-          <t>intelligenza artificiale</t>
-        </is>
-      </c>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>coding analogico</t>
-        </is>
-      </c>
-      <c r="BO2" t="inlineStr">
-        <is>
-          <t>costruzione mappe</t>
-        </is>
-      </c>
-      <c r="BP2" t="inlineStr">
-        <is>
-          <t>conversazione collaborativa / collaborazione</t>
-        </is>
-      </c>
-      <c r="BQ2" t="inlineStr">
-        <is>
-          <t>pensiero critico</t>
-        </is>
-      </c>
-      <c r="BR2" t="inlineStr">
-        <is>
-          <t>pensiero creativo</t>
-        </is>
-      </c>
-      <c r="BS2" t="inlineStr">
-        <is>
-          <t>rianalizzare</t>
-        </is>
-      </c>
-      <c r="BT2" t="inlineStr">
-        <is>
-          <t>pensiero computazionale</t>
-        </is>
-      </c>
-      <c r="BU2" t="inlineStr">
-        <is>
-          <t>risoluzione di problemi</t>
-        </is>
-      </c>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>videotutorial</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>pianificazione</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr">
-        <is>
-          <t>uso della tecnologia2</t>
         </is>
       </c>
       <c r="BY2" t="inlineStr">
@@ -4321,7 +4321,7 @@
       </c>
       <c r="CN2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> comprensione dei comandi di progrmmazione</t>
+          <t>comprensione dei comandi di programmazione</t>
         </is>
       </c>
       <c r="CO2" t="inlineStr">
@@ -6332,7 +6332,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>osservazione, memoria, analisi</t>
+          <t>osservazione/ memoria/ analisi</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">

</xml_diff>